<commit_message>
data: add HARDCORE TANO*C Pack songs
</commit_message>
<xml_diff>
--- a/data/input/kalpa-songs.xlsx
+++ b/data/input/kalpa-songs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aqua_\git\kalpa-selection\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5891FE8-288E-4872-8054-D8E6DED1533E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B7CFCA6-6EBB-4F09-9C41-F873A7E8C46C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-17295" yWindow="705" windowWidth="17235" windowHeight="14070" xr2:uid="{B18DF0BD-955E-4CF1-A738-32182884837D}"/>
+    <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" xr2:uid="{B18DF0BD-955E-4CF1-A738-32182884837D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="534">
   <si>
     <t>id</t>
   </si>
@@ -2228,6 +2228,70 @@
   </si>
   <si>
     <t>ORIGINAL</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Lost Codex</t>
+  </si>
+  <si>
+    <t>Gram VS DJ Genki</t>
+  </si>
+  <si>
+    <t>Prism Journey</t>
+  </si>
+  <si>
+    <t>Kobaryo</t>
+  </si>
+  <si>
+    <t>BUDDY MOODY</t>
+  </si>
+  <si>
+    <t>P*Light</t>
+  </si>
+  <si>
+    <t>FEEL LUV</t>
+  </si>
+  <si>
+    <t>USAO</t>
+  </si>
+  <si>
+    <t>MEGATON KICK</t>
+  </si>
+  <si>
+    <t>Everybody Say HARDCORE TANO*C</t>
+  </si>
+  <si>
+    <t>DJ Noriken</t>
+  </si>
+  <si>
+    <t>Caduceus</t>
+  </si>
+  <si>
+    <t>Gram &amp; RoughSketch</t>
+  </si>
+  <si>
+    <t>ALiVE</t>
+  </si>
+  <si>
+    <t>REDALiCE</t>
+  </si>
+  <si>
+    <t>RAV#GIRL</t>
+  </si>
+  <si>
+    <t>Srav3R</t>
+  </si>
+  <si>
+    <t>Chartreuse Green</t>
+  </si>
+  <si>
+    <t>BATTLE NO.1</t>
+  </si>
+  <si>
+    <t>TANO*C Sound Team</t>
+  </si>
+  <si>
+    <t>HARDCORE TANO*C Pack</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2683,7 +2747,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F48EBC91-EB0A-4513-A427-E3024C547FB9}">
-  <dimension ref="A1:H283"/>
+  <dimension ref="A1:H294"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="5.125" bestFit="1" customWidth="1"/>
@@ -9205,6 +9269,259 @@
         <v>16</v>
       </c>
     </row>
+    <row r="284" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A284">
+        <v>283</v>
+      </c>
+      <c r="B284" t="s">
+        <v>513</v>
+      </c>
+      <c r="C284" t="s">
+        <v>514</v>
+      </c>
+      <c r="D284" t="s">
+        <v>533</v>
+      </c>
+      <c r="E284">
+        <v>7</v>
+      </c>
+      <c r="F284">
+        <v>13</v>
+      </c>
+      <c r="G284">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="285" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A285">
+        <v>284</v>
+      </c>
+      <c r="B285" t="s">
+        <v>515</v>
+      </c>
+      <c r="C285" t="s">
+        <v>516</v>
+      </c>
+      <c r="D285" t="s">
+        <v>533</v>
+      </c>
+      <c r="E285">
+        <v>10</v>
+      </c>
+      <c r="F285">
+        <v>15</v>
+      </c>
+      <c r="G285">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="286" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A286">
+        <v>285</v>
+      </c>
+      <c r="B286" t="s">
+        <v>517</v>
+      </c>
+      <c r="C286" t="s">
+        <v>518</v>
+      </c>
+      <c r="D286" t="s">
+        <v>533</v>
+      </c>
+      <c r="E286">
+        <v>6</v>
+      </c>
+      <c r="F286">
+        <v>12</v>
+      </c>
+      <c r="G286">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="287" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A287">
+        <v>286</v>
+      </c>
+      <c r="B287" t="s">
+        <v>519</v>
+      </c>
+      <c r="C287" t="s">
+        <v>520</v>
+      </c>
+      <c r="D287" t="s">
+        <v>533</v>
+      </c>
+      <c r="E287">
+        <v>8</v>
+      </c>
+      <c r="F287">
+        <v>14</v>
+      </c>
+      <c r="G287">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="288" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A288">
+        <v>287</v>
+      </c>
+      <c r="B288" t="s">
+        <v>521</v>
+      </c>
+      <c r="C288" t="s">
+        <v>160</v>
+      </c>
+      <c r="D288" t="s">
+        <v>533</v>
+      </c>
+      <c r="E288">
+        <v>7</v>
+      </c>
+      <c r="F288">
+        <v>12</v>
+      </c>
+      <c r="G288">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="289" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A289">
+        <v>288</v>
+      </c>
+      <c r="B289" t="s">
+        <v>522</v>
+      </c>
+      <c r="C289" t="s">
+        <v>523</v>
+      </c>
+      <c r="D289" t="s">
+        <v>533</v>
+      </c>
+      <c r="E289">
+        <v>8</v>
+      </c>
+      <c r="F289">
+        <v>12</v>
+      </c>
+      <c r="G289">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="290" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A290">
+        <v>289</v>
+      </c>
+      <c r="B290" t="s">
+        <v>524</v>
+      </c>
+      <c r="C290" t="s">
+        <v>525</v>
+      </c>
+      <c r="D290" t="s">
+        <v>533</v>
+      </c>
+      <c r="E290">
+        <v>10</v>
+      </c>
+      <c r="F290">
+        <v>15</v>
+      </c>
+      <c r="G290">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="291" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A291">
+        <v>290</v>
+      </c>
+      <c r="B291" t="s">
+        <v>526</v>
+      </c>
+      <c r="C291" t="s">
+        <v>527</v>
+      </c>
+      <c r="D291" t="s">
+        <v>533</v>
+      </c>
+      <c r="E291">
+        <v>5</v>
+      </c>
+      <c r="F291">
+        <v>11</v>
+      </c>
+      <c r="G291">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="292" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A292">
+        <v>291</v>
+      </c>
+      <c r="B292" t="s">
+        <v>528</v>
+      </c>
+      <c r="C292" t="s">
+        <v>529</v>
+      </c>
+      <c r="D292" t="s">
+        <v>533</v>
+      </c>
+      <c r="E292">
+        <v>6</v>
+      </c>
+      <c r="F292">
+        <v>11</v>
+      </c>
+      <c r="G292">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="293" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A293">
+        <v>292</v>
+      </c>
+      <c r="B293" t="s">
+        <v>530</v>
+      </c>
+      <c r="C293" t="s">
+        <v>34</v>
+      </c>
+      <c r="D293" t="s">
+        <v>533</v>
+      </c>
+      <c r="E293">
+        <v>6</v>
+      </c>
+      <c r="F293">
+        <v>11</v>
+      </c>
+      <c r="G293">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="294" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A294">
+        <v>293</v>
+      </c>
+      <c r="B294" t="s">
+        <v>531</v>
+      </c>
+      <c r="C294" t="s">
+        <v>532</v>
+      </c>
+      <c r="D294" t="s">
+        <v>533</v>
+      </c>
+      <c r="E294">
+        <v>7</v>
+      </c>
+      <c r="F294">
+        <v>13</v>
+      </c>
+      <c r="G294">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H283" xr:uid="{F48EBC91-EB0A-4513-A427-E3024C547FB9}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H283">

</xml_diff>